<commit_message>
versao estavel com base relacional
</commit_message>
<xml_diff>
--- a/Simulador/dash.xlsx
+++ b/Simulador/dash.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/db44bf30ba5480d8/Documentos/Python Scripts/Fantasy/Simulador/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="208" documentId="8_{32D250B9-44B0-4D6A-89C9-E8E8B0ED30B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1BE239AA-C7F0-4210-9D12-63BCFBDB400E}"/>
+  <xr:revisionPtr revIDLastSave="241" documentId="8_{32D250B9-44B0-4D6A-89C9-E8E8B0ED30B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{878CB373-F6CD-4992-BD81-68DDA387FBC1}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{3A1DF636-5ABD-4BA5-9760-0119E916B26D}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{3A1DF636-5ABD-4BA5-9760-0119E916B26D}"/>
   </bookViews>
   <sheets>
     <sheet name="players" sheetId="1" r:id="rId1"/>
@@ -1500,6 +1500,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>